<commit_message>
Caracterización: personas únicas en estadísticas, encabezado institucional en Excel, plan de desarrollo (importador) y optimización del consolidado
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/templates/FO-PDD-19.xlsx
+++ b/resources/templates/FO-PDD-19.xlsx
@@ -5259,7 +5259,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CF1043638"/>
+  <dimension ref="A1:CF600"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.08984375" style="66" bestFit="1" customWidth="1"/>
@@ -19828,96 +19828,6 @@
         <v>42</v>
       </c>
       <c r="D334" s="64"/>
-    </row>
-    <row r="1043621" spans="5:10" ht="13" x14ac:dyDescent="0.3">
-      <c r="E1043621" s="69" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1043621" s="69"/>
-      <c r="G1043621" s="69"/>
-      <c r="H1043621" s="69"/>
-      <c r="I1043621" s="69"/>
-      <c r="J1043621" s="69"/>
-    </row>
-    <row r="1043622" spans="5:10" x14ac:dyDescent="0.25">
-      <c r="E1043622" s="66" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1043623" spans="5:10" x14ac:dyDescent="0.25">
-      <c r="E1043623" s="66" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="1043624" spans="5:10" x14ac:dyDescent="0.25">
-      <c r="E1043624" s="66" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1043625" spans="5:10" x14ac:dyDescent="0.25">
-      <c r="E1043625" s="66" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="1043626" spans="5:10" x14ac:dyDescent="0.25">
-      <c r="E1043626" s="66" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="1043627" spans="5:10" x14ac:dyDescent="0.25">
-      <c r="E1043627" s="66" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="1043628" spans="5:10" x14ac:dyDescent="0.25">
-      <c r="E1043628" s="66" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="1043629" spans="5:10" x14ac:dyDescent="0.25">
-      <c r="E1043629" s="66" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="1043632" spans="5:10" ht="13" x14ac:dyDescent="0.3">
-      <c r="E1043632" s="69" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1043632" s="69"/>
-      <c r="G1043632" s="69"/>
-      <c r="H1043632" s="69"/>
-      <c r="I1043632" s="69"/>
-      <c r="J1043632" s="69"/>
-    </row>
-    <row r="1043633" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E1043633" s="66" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="1043634" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E1043634" s="66" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="1043635" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E1043635" s="66" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="1043636" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E1043636" s="66" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="1043637" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E1043637" s="66" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="1043638" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E1043638" s="66" t="s">
-        <v>6</v>
-      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="BX15:BX99">

</xml_diff>